<commit_message>
major update, codebooks to codebook folder, 10-05 update to paper, data cleaning combined with scoring, all data from cleaning file
</commit_message>
<xml_diff>
--- a/codebook/codebook_df_analysis.xlsx
+++ b/codebook/codebook_df_analysis.xlsx
@@ -1,23 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView activeTab="0" firstSheet="0" windowHeight="13125" windowWidth="13125" xWindow="0" yWindow="0"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -42,13 +52,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
@@ -63,44 +77,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -127,32 +141,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -179,24 +175,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -208,202 +186,206 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:G108"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G112"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>pos</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>col_type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>levels</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>value_labels</t>
         </is>
@@ -431,16 +413,6 @@
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -463,16 +435,6 @@
       </c>
       <c r="E3">
         <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="4">
@@ -497,16 +459,6 @@
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -530,16 +482,6 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -563,16 +505,6 @@
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -596,16 +528,6 @@
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -629,16 +551,6 @@
       <c r="E8">
         <v>0</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -662,16 +574,6 @@
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -695,16 +597,6 @@
       <c r="E10">
         <v>3</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -728,16 +620,6 @@
       <c r="E11">
         <v>3</v>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -761,16 +643,6 @@
       <c r="E12">
         <v>3</v>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -794,16 +666,6 @@
       <c r="E13">
         <v>0</v>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -821,21 +683,11 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>chr</t>
+          <t>fct</t>
         </is>
       </c>
       <c r="E14">
         <v>0</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="15">
@@ -844,31 +696,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>motivation</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Social motivation</t>
+          <t>structure_num</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>chr</t>
+          <t>dbl</t>
         </is>
       </c>
       <c r="E15">
         <v>0</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="16">
@@ -877,31 +714,21 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>which_letter</t>
+          <t>motivation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>which letter</t>
+          <t>Social motivation</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>chr</t>
+          <t>fct</t>
         </is>
       </c>
       <c r="E16">
         <v>0</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="17">
@@ -910,32 +737,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>q7_3_1</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [25%]   The grave is not located in the northwestern part of the cemetery</t>
+          <t>motivation_prosocial</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>dbl+lbl</t>
+          <t>dbl</t>
         </is>
       </c>
       <c r="E17">
         <v>0</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="18">
@@ -944,32 +755,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>q7_3_2</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [25%]   The person buried there died before 1776</t>
+          <t>motivation_hybrid</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>dbl+lbl</t>
+          <t>dbl</t>
         </is>
       </c>
       <c r="E18">
         <v>0</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="19">
@@ -978,32 +773,21 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>q7_3_3</t>
+          <t>which_letter</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [25%]   The person buried there did not die in autumn</t>
+          <t>which letter</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>dbl+lbl</t>
+          <t>chr</t>
         </is>
       </c>
       <c r="E19">
         <v>0</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="20">
@@ -1012,13 +796,13 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>q7_3_4</t>
+          <t>q7_3_1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [25%]   The tombstone does not have any religious symbols, nature symbols, or images engraved on it</t>
+[% of Graves excluded]       Clue - [25%]   The grave is not located in the northwestern part of the cemetery</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1028,16 +812,6 @@
       </c>
       <c r="E20">
         <v>0</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="21">
@@ -1046,13 +820,13 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>q7_3_5</t>
+          <t>q7_3_2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [25%]   The inscription does not include “beloved father” on it</t>
+[% of Graves excluded]       Clue - [25%]   The person buried there died before 1776</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1062,16 +836,6 @@
       </c>
       <c r="E21">
         <v>0</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="22">
@@ -1080,13 +844,13 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>q7_3_6</t>
+          <t>q7_3_3</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [1%]    The person buried there lived fewer than 100 years</t>
+[% of Graves excluded]       Clue - [25%]   The person buried there did not die in autumn</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1096,16 +860,6 @@
       </c>
       <c r="E22">
         <v>0</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="23">
@@ -1114,13 +868,13 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>q7_3_7</t>
+          <t>q7_3_4</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [1%]    The person buried there died of natural causes</t>
+[% of Graves excluded]       Clue - [25%]   The tombstone does not have any religious symbols, nature symbols, or images engraved on it</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1130,16 +884,6 @@
       </c>
       <c r="E23">
         <v>0</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="24">
@@ -1148,13 +892,13 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>q7_3_8</t>
+          <t>q7_3_5</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [1%]    The person buried there was a monk</t>
+[% of Graves excluded]       Clue - [25%]   The inscription does not include “beloved father” on it</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1164,16 +908,6 @@
       </c>
       <c r="E24">
         <v>0</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="25">
@@ -1182,13 +916,13 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>q7_3_9</t>
+          <t>q7_3_6</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [1%]    The tombstone does not involve a statue</t>
+[% of Graves excluded]       Clue - [1%]    The person buried there lived fewer than 100 years</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1198,16 +932,6 @@
       </c>
       <c r="E25">
         <v>0</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="26">
@@ -1216,13 +940,13 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>q7_3_10</t>
+          <t>q7_3_7</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>CHURCH'S PUBLIC LETTER
-[% of Graves excluded]       Clue - [1%]    The grave is not located within 50 yards of the current grounds keepers shed</t>
+[% of Graves excluded]       Clue - [1%]    The person buried there died of natural causes</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1232,16 +956,6 @@
       </c>
       <c r="E26">
         <v>0</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="27">
@@ -1250,13 +964,13 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>q7_4_1</t>
+          <t>q7_3_8</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [25%]   The name of the person ends in "-us"</t>
+          <t>CHURCH'S PUBLIC LETTER
+[% of Graves excluded]       Clue - [1%]    The person buried there was a monk</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1266,16 +980,6 @@
       </c>
       <c r="E27">
         <v>0</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="28">
@@ -1284,13 +988,13 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>q7_4_2</t>
+          <t>q7_3_9</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [25%]   The person buried there was not an orphan</t>
+          <t>CHURCH'S PUBLIC LETTER
+[% of Graves excluded]       Clue - [1%]    The tombstone does not involve a statue</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1300,16 +1004,6 @@
       </c>
       <c r="E28">
         <v>0</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="29">
@@ -1318,13 +1012,13 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>q7_4_3</t>
+          <t>q7_3_10</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [25%]   The grave is not on the hill of the cemetery</t>
+          <t>CHURCH'S PUBLIC LETTER
+[% of Graves excluded]       Clue - [1%]    The grave is not located within 50 yards of the current grounds keepers shed</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1334,16 +1028,6 @@
       </c>
       <c r="E29">
         <v>0</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="30">
@@ -1352,13 +1036,13 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>q7_4_4</t>
+          <t>q7_4_1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [25%]   The person buried there was not born in springtime</t>
+[% of Graves excluded]       Clue - [25%]   The name of the person ends in "-us"</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1368,16 +1052,6 @@
       </c>
       <c r="E30">
         <v>0</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="31">
@@ -1386,13 +1060,13 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>q7_4_5</t>
+          <t>q7_4_2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
           <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [25%]   The grave is not located in the southeastern part of the cemetery</t>
+[% of Graves excluded]       Clue - [25%]   The person buried there was not an orphan</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1402,16 +1076,6 @@
       </c>
       <c r="E31">
         <v>0</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="32">
@@ -1420,13 +1084,13 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>q7_4_6</t>
+          <t>q7_4_3</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
           <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [1%]    The person is not buried a mausoleum</t>
+[% of Graves excluded]       Clue - [25%]   The grave is not on the hill of the cemetery</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1436,16 +1100,6 @@
       </c>
       <c r="E32">
         <v>0</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="33">
@@ -1454,13 +1108,13 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>q7_4_7</t>
+          <t>q7_4_4</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
           <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [1%]    The tombstone includes the person's first name, last name, and date of death</t>
+[% of Graves excluded]       Clue - [25%]   The person buried there was not born in springtime</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1470,16 +1124,6 @@
       </c>
       <c r="E33">
         <v>0</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="34">
@@ -1488,13 +1132,13 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>q7_4_8</t>
+          <t>q7_4_5</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [1%]    The grave is not located next to the old oak tree</t>
+[% of Graves excluded]       Clue - [25%]   The grave is not located in the southeastern part of the cemetery</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1504,16 +1148,6 @@
       </c>
       <c r="E34">
         <v>0</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="35">
@@ -1522,13 +1156,13 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>q7_4_9</t>
+          <t>q7_4_6</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
           <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [1%]    The treasure is not in grave 84, 85, 86, or 87</t>
+[% of Graves excluded]       Clue - [1%]    The person is not buried a mausoleum</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1538,16 +1172,6 @@
       </c>
       <c r="E35">
         <v>0</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="36">
@@ -1556,13 +1180,13 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>q7_4_10</t>
+          <t>q7_4_7</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
           <t>ONLY [Field-which%20letter]
-[% of Graves excluded]       Clue - [1%]    The tombstone is made of white marble</t>
+[% of Graves excluded]       Clue - [1%]    The tombstone includes the person's first name, last name, and date of death</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1572,16 +1196,6 @@
       </c>
       <c r="E36">
         <v>0</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2, 1, 3</t>
-        </is>
       </c>
     </row>
     <row r="37">
@@ -1590,12 +1204,13 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>q9_1_1</t>
+          <t>q7_4_8</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>STRATEGIES - I did not think much about what I shared.</t>
+          <t>ONLY [Field-which%20letter]
+[% of Graves excluded]       Clue - [1%]    The grave is not located next to the old oak tree</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1604,17 +1219,7 @@
         </is>
       </c>
       <c r="E37">
-        <v>2</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1623,12 +1228,13 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>q9_1_2</t>
+          <t>q7_4_9</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>STRATEGIES - I shared what I thought was interesting.</t>
+          <t>ONLY [Field-which%20letter]
+[% of Graves excluded]       Clue - [1%]    The treasure is not in grave 84, 85, 86, or 87</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1637,17 +1243,7 @@
         </is>
       </c>
       <c r="E38">
-        <v>2</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1656,12 +1252,13 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>q9_1_3</t>
+          <t>q7_4_10</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>STRATEGIES - I just shared everything.</t>
+          <t>ONLY [Field-which%20letter]
+[% of Graves excluded]       Clue - [1%]    The tombstone is made of white marble</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1670,17 +1267,7 @@
         </is>
       </c>
       <c r="E39">
-        <v>2</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1689,12 +1276,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>q9_1_4</t>
+          <t>q9_1_1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>STRATEGIES - I tried to share very little information.</t>
+          <t>STRATEGIES - I did not think much about what I shared.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1704,16 +1291,6 @@
       </c>
       <c r="E40">
         <v>2</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="41">
@@ -1722,12 +1299,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>q9_1_5</t>
+          <t>q9_1_2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>STRATEGIES - I tried to share as much information as possible.</t>
+          <t>STRATEGIES - I shared what I thought was interesting.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1737,16 +1314,6 @@
       </c>
       <c r="E41">
         <v>2</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="42">
@@ -1755,12 +1322,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>q9_1_6</t>
+          <t>q9_1_3</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>STRATEGIES - I tried to share information that ruled out more graves.</t>
+          <t>STRATEGIES - I just shared everything.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1770,16 +1337,6 @@
       </c>
       <c r="E42">
         <v>2</v>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="43">
@@ -1788,12 +1345,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>q9_1_7</t>
+          <t>q9_1_4</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>STRATEGIES - I focused more on sharing information that ruled out fewer graves.</t>
+          <t>STRATEGIES - I tried to share very little information.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1803,16 +1360,6 @@
       </c>
       <c r="E43">
         <v>2</v>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="44">
@@ -1821,12 +1368,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>q9_1_8</t>
+          <t>q9_1_5</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>STRATEGIES - I focused on sharing information that everyone already had access to.</t>
+          <t>STRATEGIES - I tried to share as much information as possible.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1836,16 +1383,6 @@
       </c>
       <c r="E44">
         <v>2</v>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="45">
@@ -1854,12 +1391,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>q9_1_9</t>
+          <t>q9_1_6</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>STRATEGIES - I tried to share information that others likely did not know yet.</t>
+          <t>STRATEGIES - I tried to share information that ruled out more graves.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1869,16 +1406,6 @@
       </c>
       <c r="E45">
         <v>2</v>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="46">
@@ -1887,12 +1414,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>q9_1_10</t>
+          <t>q9_1_7</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>STRATEGIES - I tried to share information that ruled out more graves and others did not know.</t>
+          <t>STRATEGIES - I focused more on sharing information that ruled out fewer graves.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1902,16 +1429,6 @@
       </c>
       <c r="E46">
         <v>2</v>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="47">
@@ -1920,12 +1437,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>q9_1_11</t>
+          <t>q9_1_8</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>STRATEGIES - I tried to share information that ruled out fewer graves and others did not know.</t>
+          <t>STRATEGIES - I focused on sharing information that everyone already had access to.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1935,16 +1452,6 @@
       </c>
       <c r="E47">
         <v>2</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="48">
@@ -1953,12 +1460,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>q9_1_12</t>
+          <t>q9_1_9</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>STRATEGIES - I tried to share information that ruled out more graves and others already knew.</t>
+          <t>STRATEGIES - I tried to share information that others likely did not know yet.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1968,16 +1475,6 @@
       </c>
       <c r="E48">
         <v>2</v>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="49">
@@ -1986,12 +1483,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>q9_1_13</t>
+          <t>q9_1_10</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>STRATEGIES - I tried to share information that ruled out fewer graves and others already knew.</t>
+          <t>STRATEGIES - I tried to share information that ruled out more graves and others did not know.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2001,16 +1498,6 @@
       </c>
       <c r="E49">
         <v>2</v>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="50">
@@ -2019,12 +1506,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>q10_1_1</t>
+          <t>q9_1_11</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>COOPERATION - During the task, I had to compete against everyone to succeed.</t>
+          <t>STRATEGIES - I tried to share information that ruled out fewer graves and others did not know.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2034,16 +1521,6 @@
       </c>
       <c r="E50">
         <v>2</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="51">
@@ -2052,12 +1529,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>q10_1_2</t>
+          <t>q9_1_12</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>COOPERATION - During the task, I was trying to get more clues for myself.</t>
+          <t>STRATEGIES - I tried to share information that ruled out more graves and others already knew.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2067,16 +1544,6 @@
       </c>
       <c r="E51">
         <v>2</v>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="52">
@@ -2085,12 +1552,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>q10_1_3</t>
+          <t>q9_1_13</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>COOPERATION - During the task, I was especially motivated to solve the task for myself.</t>
+          <t>STRATEGIES - I tried to share information that ruled out fewer graves and others already knew.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2100,16 +1567,6 @@
       </c>
       <c r="E52">
         <v>2</v>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="53">
@@ -2118,12 +1575,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>q10_1_4</t>
+          <t>q10_1_1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>COOPERATION - During the task, it was important for me to solve the task first.</t>
+          <t>COOPERATION - During the task, I had to compete against everyone to succeed.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2133,16 +1590,6 @@
       </c>
       <c r="E53">
         <v>2</v>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="54">
@@ -2151,12 +1598,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>q10_1_5</t>
+          <t>q10_1_2</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>COOPERATION - During the task, I wanted to help everyone so we could solve the task.</t>
+          <t>COOPERATION - During the task, I was trying to get more clues for myself.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2166,16 +1613,6 @@
       </c>
       <c r="E54">
         <v>2</v>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="55">
@@ -2184,12 +1621,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>q10_1_6</t>
+          <t>q10_1_3</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>COOPERATION - During the task, I wanted to share clues with everyone.</t>
+          <t>COOPERATION - During the task, I was especially motivated to solve the task for myself.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2199,16 +1636,6 @@
       </c>
       <c r="E55">
         <v>2</v>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="56">
@@ -2217,12 +1644,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>q10_1_7</t>
+          <t>q10_1_4</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>COOPERATION - During the task, I tried to help solve the task regardless of who found the solution first.</t>
+          <t>COOPERATION - During the task, it was important for me to solve the task first.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2232,16 +1659,6 @@
       </c>
       <c r="E56">
         <v>2</v>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="57">
@@ -2250,12 +1667,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>q10_1_8</t>
+          <t>q10_1_5</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>COOPERATION - During the task, increasing everyone’s performance would increase my own chances of success.</t>
+          <t>COOPERATION - During the task, I wanted to help everyone so we could solve the task.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2265,16 +1682,6 @@
       </c>
       <c r="E57">
         <v>2</v>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="58">
@@ -2283,12 +1690,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>q11_1_1</t>
+          <t>q10_1_6</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to manipulate others to get my way.</t>
+          <t>COOPERATION - During the task, I wanted to share clues with everyone.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2298,16 +1705,6 @@
       </c>
       <c r="E58">
         <v>2</v>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="59">
@@ -2316,12 +1713,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>q11_1_2</t>
+          <t>q10_1_7</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>DOZEN - I have used deceit or lied to get my way.</t>
+          <t>COOPERATION - During the task, I tried to help solve the task regardless of who found the solution first.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2331,16 +1728,6 @@
       </c>
       <c r="E59">
         <v>2</v>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="60">
@@ -2349,12 +1736,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>q11_1_3</t>
+          <t>q10_1_8</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>DOZEN - I have used flattery to get my way.</t>
+          <t>COOPERATION - During the task, increasing everyone’s performance would increase my own chances of success.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2364,16 +1751,6 @@
       </c>
       <c r="E60">
         <v>2</v>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="61">
@@ -2382,12 +1759,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>q11_1_4</t>
+          <t>q11_1_1</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to exploit others towards my own end.</t>
+          <t>DOZEN - I tend to manipulate others to get my way.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2397,16 +1774,6 @@
       </c>
       <c r="E61">
         <v>2</v>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="62">
@@ -2415,12 +1782,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>q11_1_5</t>
+          <t>q11_1_2</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to lack remorse.</t>
+          <t>DOZEN - I have used deceit or lied to get my way.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2430,16 +1797,6 @@
       </c>
       <c r="E62">
         <v>2</v>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="63">
@@ -2448,12 +1805,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>q11_1_6</t>
+          <t>q11_1_3</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to be unconcerned with the morality of my actions.</t>
+          <t>DOZEN - I have used flattery to get my way.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2463,16 +1820,6 @@
       </c>
       <c r="E63">
         <v>2</v>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="64">
@@ -2481,12 +1828,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>q11_1_7</t>
+          <t>q11_1_4</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to be callous or insensitive</t>
+          <t>DOZEN - I tend to exploit others towards my own end.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2496,16 +1843,6 @@
       </c>
       <c r="E64">
         <v>2</v>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="65">
@@ -2514,12 +1851,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>q11_1_8</t>
+          <t>q11_1_5</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to be cynical.</t>
+          <t>DOZEN - I tend to lack remorse.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2529,16 +1866,6 @@
       </c>
       <c r="E65">
         <v>2</v>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="66">
@@ -2547,12 +1874,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>q11_1_9</t>
+          <t>q11_1_6</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to want others to admire me.</t>
+          <t>DOZEN - I tend to be unconcerned with the morality of my actions.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2562,16 +1889,6 @@
       </c>
       <c r="E66">
         <v>2</v>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="67">
@@ -2580,12 +1897,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>q11_1_10</t>
+          <t>q11_1_7</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to want others to pay attention to me.</t>
+          <t>DOZEN - I tend to be callous or insensitive</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2595,16 +1912,6 @@
       </c>
       <c r="E67">
         <v>2</v>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="68">
@@ -2613,12 +1920,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>q11_1_11</t>
+          <t>q11_1_8</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to seek prestige or status.</t>
+          <t>DOZEN - I tend to be cynical.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2628,16 +1935,6 @@
       </c>
       <c r="E68">
         <v>2</v>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="69">
@@ -2646,12 +1943,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>q11_1_12</t>
+          <t>q11_1_9</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>DOZEN - I tend to expect special favors from others.</t>
+          <t>DOZEN - I tend to want others to admire me.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2661,16 +1958,6 @@
       </c>
       <c r="E69">
         <v>2</v>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="70">
@@ -2679,12 +1966,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>q12_1_1</t>
+          <t>q11_1_10</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>NEEDCOG - I would prefer complex to simple problems.</t>
+          <t>DOZEN - I tend to want others to pay attention to me.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2693,17 +1980,7 @@
         </is>
       </c>
       <c r="E70">
-        <v>1</v>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
@@ -2712,12 +1989,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>q12_1_2</t>
+          <t>q11_1_11</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>NEEDCOG - I like to have the responsibility of handling a situation that requires a lot of thinking.</t>
+          <t>DOZEN - I tend to seek prestige or status.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2726,17 +2003,7 @@
         </is>
       </c>
       <c r="E71">
-        <v>1</v>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -2745,12 +2012,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>q12_1_3</t>
+          <t>q11_1_12</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>NEEDCOG - Thinking is not my idea of fun.</t>
+          <t>DOZEN - I tend to expect special favors from others.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2759,17 +2026,7 @@
         </is>
       </c>
       <c r="E72">
-        <v>1</v>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="73">
@@ -2778,12 +2035,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>q12_1_4</t>
+          <t>q12_1_1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>NEEDCOG - I would rather do something that requires little thought than something that is sure to challenge my thinking abilities.</t>
+          <t>NEEDCOG - I would prefer complex to simple problems.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2793,16 +2050,6 @@
       </c>
       <c r="E73">
         <v>1</v>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="74">
@@ -2811,12 +2058,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>q12_1_5</t>
+          <t>q12_1_2</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>NEEDCOG - I try to anticipate and avoid situations where there is a likely chance I will have to think in depth about something.</t>
+          <t>NEEDCOG - I like to have the responsibility of handling a situation that requires a lot of thinking.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2826,16 +2073,6 @@
       </c>
       <c r="E74">
         <v>1</v>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="75">
@@ -2844,12 +2081,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>q12_1_6</t>
+          <t>q12_1_3</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>NEEDCOG - I find satisfaction in deliberating hard and for long hours.</t>
+          <t>NEEDCOG - Thinking is not my idea of fun.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2859,16 +2096,6 @@
       </c>
       <c r="E75">
         <v>1</v>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="76">
@@ -2877,12 +2104,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>q12_1_7</t>
+          <t>q12_1_4</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>NEEDCOG - I only think as hard as I have to.</t>
+          <t>NEEDCOG - I would rather do something that requires little thought than something that is sure to challenge my thinking abilities.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2892,16 +2119,6 @@
       </c>
       <c r="E76">
         <v>1</v>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="77">
@@ -2910,12 +2127,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>q12_1_8</t>
+          <t>q12_1_5</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>NEEDCOG - I prefer to think about small, daily projects than long-term ones.</t>
+          <t>NEEDCOG - I try to anticipate and avoid situations where there is a likely chance I will have to think in depth about something.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2925,16 +2142,6 @@
       </c>
       <c r="E77">
         <v>1</v>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="78">
@@ -2943,12 +2150,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>q12_1_9</t>
+          <t>q12_1_6</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>NEEDCOG - I like tasks that require little thought once I’ve learned them.</t>
+          <t>NEEDCOG - I find satisfaction in deliberating hard and for long hours.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2958,16 +2165,6 @@
       </c>
       <c r="E78">
         <v>1</v>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="79">
@@ -2976,12 +2173,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>q12_1_10</t>
+          <t>q12_1_7</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>NEEDCOG - The idea of relying on thought to make my way to the top appeals to me.</t>
+          <t>NEEDCOG - I only think as hard as I have to.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2991,16 +2188,6 @@
       </c>
       <c r="E79">
         <v>1</v>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="80">
@@ -3009,12 +2196,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>q12_1_11</t>
+          <t>q12_1_8</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>NEEDCOG - I really enjoy a task that involves coming up with new solutions to problems.</t>
+          <t>NEEDCOG - I prefer to think about small, daily projects than long-term ones.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3024,16 +2211,6 @@
       </c>
       <c r="E80">
         <v>1</v>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="81">
@@ -3042,12 +2219,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>q12_1_12</t>
+          <t>q12_1_9</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>NEEDCOG - Learning new ways to think doesn’t excite me very much.</t>
+          <t>NEEDCOG - I like tasks that require little thought once I’ve learned them.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3057,16 +2234,6 @@
       </c>
       <c r="E81">
         <v>1</v>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="82">
@@ -3075,12 +2242,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>q12_1_13</t>
+          <t>q12_1_10</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>NEEDCOG - I prefer my life to be filled with puzzles that I must solve.</t>
+          <t>NEEDCOG - The idea of relying on thought to make my way to the top appeals to me.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3090,16 +2257,6 @@
       </c>
       <c r="E82">
         <v>1</v>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="83">
@@ -3108,12 +2265,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>q12_1_14</t>
+          <t>q12_1_11</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>NEEDCOG - The notion of thinking abstractly is appealing to me.</t>
+          <t>NEEDCOG - I really enjoy a task that involves coming up with new solutions to problems.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3123,16 +2280,6 @@
       </c>
       <c r="E83">
         <v>1</v>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="84">
@@ -3141,12 +2288,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>q12_1_15</t>
+          <t>q12_1_12</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>NEEDCOG - I would prefer a task that is intellectual, difficult, and important to one that is somewhat important but does not require much thought.</t>
+          <t>NEEDCOG - Learning new ways to think doesn’t excite me very much.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3156,16 +2303,6 @@
       </c>
       <c r="E84">
         <v>1</v>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="85">
@@ -3174,12 +2311,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>q12_1_16</t>
+          <t>q12_1_13</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>NEEDCOG - I feel relief rather than satisfaction after completing a task that required a lot of mental effort.</t>
+          <t>NEEDCOG - I prefer my life to be filled with puzzles that I must solve.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3189,16 +2326,6 @@
       </c>
       <c r="E85">
         <v>1</v>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="86">
@@ -3207,12 +2334,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>q12_1_17</t>
+          <t>q12_1_14</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>NEEDCOG - It’s enough for me that something gets the job done; I don’t care how or why it works.</t>
+          <t>NEEDCOG - The notion of thinking abstractly is appealing to me.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3222,16 +2349,6 @@
       </c>
       <c r="E86">
         <v>1</v>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="87">
@@ -3240,12 +2357,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>q12_1_18</t>
+          <t>q12_1_15</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>NEEDCOG - I usually end up deliberating about issues even when they do not affect me personally.</t>
+          <t>NEEDCOG - I would prefer a task that is intellectual, difficult, and important to one that is somewhat important but does not require much thought.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3255,16 +2372,6 @@
       </c>
       <c r="E87">
         <v>1</v>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
       </c>
     </row>
     <row r="88">
@@ -3273,32 +2380,21 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>q14_2</t>
+          <t>q12_1_16</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Please let us know if you have feedback on this project.
-For example, what issues, if any, did you have any issues completing the survey? Which questions or instructions, if any, did you find confusing or unclear? If you experienced technical problems, please describe.</t>
+          <t>NEEDCOG - I feel relief rather than satisfaction after completing a task that required a lot of mental effort.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>chr</t>
+          <t>dbl+lbl</t>
         </is>
       </c>
       <c r="E88">
-        <v>0</v>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -3307,31 +2403,21 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>total_approvals</t>
+          <t>q12_1_17</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Total Prolific approvals</t>
+          <t>NEEDCOG - It’s enough for me that something gets the job done; I don’t care how or why it works.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>dbl</t>
+          <t>dbl+lbl</t>
         </is>
       </c>
       <c r="E89">
-        <v>3</v>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -3340,31 +2426,21 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>undergraduate_year_of_study</t>
+          <t>q12_1_18</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Undergraduate year of study</t>
+          <t>NEEDCOG - I usually end up deliberating about issues even when they do not affect me personally.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>fct</t>
+          <t>dbl+lbl</t>
         </is>
       </c>
       <c r="E90">
-        <v>49</v>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>1st Year, 2nd Year, 3rd Year, 4th Year, Other</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -3373,31 +2449,22 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>fluent_languages</t>
+          <t>q14_2</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Fluent languages</t>
+          <t>Please let us know if you have feedback on this project.
+For example, what issues, if any, did you have any issues completing the survey? Which questions or instructions, if any, did you find confusing or unclear? If you experienced technical problems, please describe.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>fct</t>
+          <t>chr</t>
         </is>
       </c>
       <c r="E91">
-        <v>3</v>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>Arabic, English, Cantonese, English, Mandarin, Chinese, English, Chinese, English, Mandarin, Somali, Swahili, English, English, Arabic, English, Bengali, English, Chinese, English, French, English, German, English, Hungarian, English, Mandarin, English, Other, English, Portuguese, English, Russian, English, Spanish, English, Swahili, English, Urdu, Farsi, English, Japanese, English, Spanish, Korean, English, Portuguese, English, Romanian, Spanish, English, Russian, Ukrainian, English, Spanish, English, Telugu, English</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -3406,31 +2473,21 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>relationship_marital_status</t>
+          <t>total_approvals</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Relationship or marital status</t>
+          <t>Total Prolific approvals</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>fct</t>
+          <t>dbl</t>
         </is>
       </c>
       <c r="E92">
         <v>3</v>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>Divorced, Engaged, In a relationship, Married, Never married, Single</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="93">
@@ -3439,12 +2496,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>undergraduate_year_of_study</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Undergraduate year of study</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3453,17 +2510,7 @@
         </is>
       </c>
       <c r="E93">
-        <v>6</v>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>Man (including Trans Male/Trans Man), Non-binary (would like to give more detail), Woman (including Trans Female/Trans Woman)</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>49</v>
       </c>
     </row>
     <row r="94">
@@ -3472,12 +2519,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>current_u_s_state_of_residence</t>
+          <t>fluent_languages</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Current U.S. state of residence</t>
+          <t>Fluent languages</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3487,16 +2534,6 @@
       </c>
       <c r="E94">
         <v>3</v>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Alabama (AL), Arizona (AZ), Arkansas (AR), California (CA), Colorado (CO), Connecticut (CT), Delaware (DE), Florida (FL), Georgia (GA), Hawaii (HI), Idaho (ID), Illinois (IL), Indiana (IN), Iowa (IA), Kansas (KS), Kentucky (KY), Louisiana (LA), Maryland (MD), Massachusetts (MA), Michigan (MI), Minnesota (MN), Mississippi (MS), Missouri (MO), Nevada (NV), New Jersey (NJ), New York (NY), North Carolina (NC), Ohio (OH), Oklahoma (OK), Oregon (OR), Pennsylvania (PA), Rhode Island (RI), South Carolina (SC), Tennessee (TN), Texas (TX), Virginia (VA), Washington (WA), Wisconsin (WI), Wyoming (WY)</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="95">
@@ -3505,31 +2542,21 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>household_income_usd_us_participants_only</t>
+          <t>relationship_marital_status</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Household income (USD; U.S. participants only)</t>
+          <t>Relationship or marital status</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>ord</t>
+          <t>fct</t>
         </is>
       </c>
       <c r="E95">
-        <v>95</v>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>Less than $10000, $10000–$15999, $16000–$19999, $20000–$24999, $25000–$29999, $30000–$34999, $35000–$39999, $40000–$49999, $50000–$59999, $60000–$74999, $75000–$99999, $100000–$149999, More than $150000</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="96">
@@ -3538,12 +2565,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>highest_level_of_education_completed_by_parents</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Highest level of education completed by parents</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3552,17 +2579,7 @@
         </is>
       </c>
       <c r="E96">
-        <v>3</v>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>No formal qualifications, Secondary education (e.g. GED/GCSE), High school diploma / A-Levels / Community college, Undergraduate degree (BA/BSc/Other), Graduate degree (MA,MSc/MPhil/Other), Doctorate degree (PhD/other), Don't know, Not applicable / Prefer not to say</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>6</v>
       </c>
     </row>
     <row r="97">
@@ -3571,31 +2588,21 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>personal_income_usd_us_participants_only</t>
+          <t>current_u_s_state_of_residence</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Personal income (USD; U.S. participants only)</t>
+          <t>Current U.S. state of residence</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>ord</t>
+          <t>fct</t>
         </is>
       </c>
       <c r="E97">
-        <v>230</v>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>Less than $10000, $10000–$15999, $16000–$19999, $20000–$24999, $25000–$29999, $30000–$34999, $35000–$39999, $40000–$49999, $50000–$59999, $60000–$74999, $75000–$99999, $100000–$149999, More than $150000, Rather not say</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="98">
@@ -3604,31 +2611,21 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>age</t>
+          <t>household_income_usd_us_participants_only</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Age</t>
+          <t>Household income (USD; U.S. participants only)</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>dbl</t>
+          <t>ord</t>
         </is>
       </c>
       <c r="E98">
-        <v>3</v>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>95</v>
       </c>
     </row>
     <row r="99">
@@ -3637,12 +2634,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>highest_level_of_education_completed_by_parents</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Highest level of education completed by parents</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3652,16 +2649,6 @@
       </c>
       <c r="E99">
         <v>3</v>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>Female, Male</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="100">
@@ -3670,31 +2657,21 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ethnicity_simplified</t>
+          <t>personal_income_usd_us_participants_only</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Ethnicity, simplified</t>
+          <t>Personal income (USD; U.S. participants only)</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>fct</t>
+          <t>ord</t>
         </is>
       </c>
       <c r="E100">
-        <v>6</v>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>Asian, Black, Mixed, Other, White</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>230</v>
       </c>
     </row>
     <row r="101">
@@ -3703,31 +2680,21 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>country_of_birth</t>
+          <t>age</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Country of birth</t>
+          <t>Age</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>fct</t>
+          <t>dbl</t>
         </is>
       </c>
       <c r="E101">
         <v>3</v>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>Brazil, Canada, China, Colombia, Cuba, Dominican Republic, Guyana, Haiti, Jordan, Kenya, Mexico, Nigeria, Saudi Arabia, Turkey, United Kingdom, United States, United States Minor Outlying Islands</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="102">
@@ -3736,12 +2703,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>country_of_residence</t>
+          <t>sex</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Country of residence</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3751,16 +2718,6 @@
       </c>
       <c r="E102">
         <v>3</v>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="103">
@@ -3769,31 +2726,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>nationality</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>Nationality</t>
+          <t>sex_num</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>fct</t>
+          <t>dbl</t>
         </is>
       </c>
       <c r="E103">
         <v>3</v>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>Brazil, China, Colombia, Cuba, Dominican Republic, Germany, Guyana, Haiti, Iran, Italy, Japan, Mexico, Nigeria, Puerto Rico, Turkey, United Kingdom, United States</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="104">
@@ -3802,12 +2744,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>language</t>
+          <t>ethnicity_simplified</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Primary language</t>
+          <t>Ethnicity, simplified</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3816,17 +2758,7 @@
         </is>
       </c>
       <c r="E104">
-        <v>3</v>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>Arabic, Cantonese, Chinese, English, French, Japanese, Mandarin, Portuguese, Romanian, Russian, Serbian, Spanish, Swahili, Turkish, Urdu</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>6</v>
       </c>
     </row>
     <row r="105">
@@ -3835,29 +2767,21 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>n_fluent_languages</t>
-        </is>
-      </c>
-      <c r="C105" t="e">
-        <v>#N/A</v>
+          <t>country_of_birth</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Country of birth</t>
+        </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>fct</t>
         </is>
       </c>
       <c r="E105">
         <v>3</v>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="106">
@@ -3866,11 +2790,13 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>multilingual</t>
-        </is>
-      </c>
-      <c r="C106" t="e">
-        <v>#N/A</v>
+          <t>country_of_residence</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Country of residence</t>
+        </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -3879,16 +2805,6 @@
       </c>
       <c r="E106">
         <v>3</v>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>One language, Multiple languages</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="107">
@@ -3897,12 +2813,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>student_status</t>
+          <t>nationality</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Student status</t>
+          <t>Nationality</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3912,16 +2828,6 @@
       </c>
       <c r="E107">
         <v>3</v>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>DATA_EXPIRED, No, Yes</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t/>
-        </is>
       </c>
     </row>
     <row r="108">
@@ -3930,12 +2836,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>employment_status</t>
+          <t>language</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Employment status</t>
+          <t>Primary language</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3946,20 +2852,90 @@
       <c r="E108">
         <v>3</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>Due to start a new job within the next month, Full-Time, Not in paid work (e.g. homemaker', 'retired or disabled), Other, Part-Time, Unemployed (and job seeking)</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>n_fluent_languages</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E109">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>multilingual</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>fct</t>
+        </is>
+      </c>
+      <c r="E110">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>student_status</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Student status</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>fct</t>
+        </is>
+      </c>
+      <c r="E111">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>employment_status</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Employment status</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>fct</t>
+        </is>
+      </c>
+      <c r="E112">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="1" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>